<commit_message>
WIP: BOOTH listing plan (titles, tags, price proposals)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QRNFBqosexHq3udDF3YWyM
</commit_message>
<xml_diff>
--- a/company/product/P3/dist/allergen-ichiran.xlsx
+++ b/company/product/P3/dist/allergen-ichiran.xlsx
@@ -5258,8 +5258,8 @@
     <col width="3" customWidth="1" min="28" max="28"/>
     <col width="3" customWidth="1" min="29" max="29"/>
     <col width="3" customWidth="1" min="30" max="30"/>
-    <col width="9.199999999999999" customWidth="1" min="31" max="31"/>
-    <col width="30" customWidth="1" min="32" max="32"/>
+    <col width="10.5" customWidth="1" min="31" max="31"/>
+    <col width="28.8" customWidth="1" min="32" max="32"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -12061,7 +12061,7 @@
   <pageSetup orientation="landscape" paperSize="9" scale="100"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;C&amp;10 &amp;P / &amp;N</oddFooter>
+    <oddFooter>&amp;C&amp;10 &amp;Pページ</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
WIP: QA round-1 fixes in progress (README trademark notes, P3 compat wording)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QRNFBqosexHq3udDF3YWyM
</commit_message>
<xml_diff>
--- a/company/product/P3/dist/allergen-ichiran.xlsx
+++ b/company/product/P3/dist/allergen-ichiran.xlsx
@@ -600,7 +600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:A50"/>
+  <dimension ref="A1:A49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="85" customWidth="1" min="1" max="1"/>
@@ -889,36 +889,29 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>・Google ドライブにアップロードし、「Google スプレッドシートで開く」→ ファイル →「Google スプレッドシートとして保存」。</t>
+          <t>・Google ドライブにアップロードし、ファイルを右クリック →「アプリで開く」→「Google スプレッドシート」。続けて ファイル →「Google スプレッドシートとして保存」。</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>・スマートフォンでもプルダウンから選べます（プルダウンの作成・変更はパソコンが必要です）。</t>
-        </is>
-      </c>
+      <c r="A46" s="2" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="inlineStr"/>
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>■ その他</t>
+        </is>
+      </c>
     </row>
     <row r="48">
-      <c r="A48" s="3" t="inlineStr">
-        <is>
-          <t>■ その他</t>
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>・色の付いたセル（区分・品目名・状態・お客様用シート）は自動計算です。消したり上書きしたりしないでください。シートの保護はしていません。</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
-        <is>
-          <t>・色の付いたセル（区分・品目名・状態・お客様用シート）は自動計算です。消したり上書きしたりしないでください。シートの保護はしていません。</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="inlineStr">
         <is>
           <t>・見本の店名「〇〇食堂（見本）」と3品のメニューは架空のものです。見本の ○／－ は「見本の架空データ。実際のメニューには使えない」ものです。</t>
         </is>

</xml_diff>